<commit_message>
Update image generation and SKU workflows
</commit_message>
<xml_diff>
--- a/tools/python/temu-product-sheet/data/size_specs.xlsx
+++ b/tools/python/temu-product-sheet/data/size_specs.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="15600" windowHeight="9675"/>
+    <workbookView windowWidth="23145" windowHeight="9675"/>
   </bookViews>
   <sheets>
     <sheet name="商品主表" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="119">
   <si>
     <t>宽度（cm）</t>
   </si>
@@ -74,46 +74,115 @@
     <t>申报价（￥）</t>
   </si>
   <si>
+    <t>44-50</t>
+  </si>
+  <si>
     <t>120-150</t>
   </si>
   <si>
-    <t>14-16</t>
+    <t>22-26</t>
   </si>
   <si>
     <t>151-180</t>
   </si>
   <si>
-    <t>16-18</t>
+    <t>23-27</t>
   </si>
   <si>
     <t>181-200</t>
   </si>
   <si>
-    <t>18-20</t>
+    <t>24-28</t>
   </si>
   <si>
     <t>201-230</t>
   </si>
   <si>
-    <t>20-22</t>
+    <t>24-30</t>
   </si>
   <si>
     <t>231-250</t>
   </si>
   <si>
-    <t>24-26</t>
+    <t>30-32</t>
   </si>
   <si>
     <t>251-280</t>
   </si>
   <si>
-    <t>26-28</t>
+    <t>31-36</t>
   </si>
   <si>
     <t>281-300</t>
   </si>
   <si>
+    <t>32-42</t>
+  </si>
+  <si>
+    <t>51-55</t>
+  </si>
+  <si>
+    <t>25-27</t>
+  </si>
+  <si>
     <t>28-30</t>
+  </si>
+  <si>
+    <t>32-30</t>
+  </si>
+  <si>
+    <t>30-35</t>
+  </si>
+  <si>
+    <t>35-40</t>
+  </si>
+  <si>
+    <t>38-45</t>
+  </si>
+  <si>
+    <t>56-60</t>
+  </si>
+  <si>
+    <t>24-27</t>
+  </si>
+  <si>
+    <t>26-27</t>
+  </si>
+  <si>
+    <t>28-31</t>
+  </si>
+  <si>
+    <t>32-35</t>
+  </si>
+  <si>
+    <t>33-36</t>
+  </si>
+  <si>
+    <t>36-40</t>
+  </si>
+  <si>
+    <t>40-45</t>
+  </si>
+  <si>
+    <t>61-65</t>
+  </si>
+  <si>
+    <t>28-33</t>
+  </si>
+  <si>
+    <t>66-70</t>
+  </si>
+  <si>
+    <t>33-35</t>
+  </si>
+  <si>
+    <t>35-36</t>
+  </si>
+  <si>
+    <t>38-40</t>
+  </si>
+  <si>
+    <t>41-45</t>
   </si>
   <si>
     <t>商品编号</t>
@@ -1551,11 +1620,11 @@
       </c>
     </row>
     <row r="2" s="8" customFormat="1" ht="24" customHeight="1" spans="1:7">
-      <c r="A2" s="16">
-        <v>50</v>
+      <c r="A2" s="16" t="s">
+        <v>7</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="16">
         <v>50</v>
@@ -1570,15 +1639,15 @@
         <v>320</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" s="9" customFormat="1" ht="24" customHeight="1" spans="1:7">
-      <c r="A3" s="16">
-        <v>50</v>
+      <c r="A3" s="16" t="s">
+        <v>7</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" s="16">
         <v>50</v>
@@ -1593,15 +1662,15 @@
         <v>340</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" s="9" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A4" s="16">
-        <v>50</v>
+      <c r="A4" s="16" t="s">
+        <v>7</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="16">
         <v>50</v>
@@ -1616,15 +1685,15 @@
         <v>360</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" s="9" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A5" s="16">
-        <v>50</v>
+      <c r="A5" s="16" t="s">
+        <v>7</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" s="16">
         <v>50</v>
@@ -1639,15 +1708,15 @@
         <v>380</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" s="9" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A6" s="16">
-        <v>50</v>
+      <c r="A6" s="16" t="s">
+        <v>7</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" s="16">
         <v>50</v>
@@ -1662,15 +1731,15 @@
         <v>400</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" s="9" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A7" s="16">
-        <v>50</v>
+      <c r="A7" s="16" t="s">
+        <v>7</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" s="16">
         <v>50</v>
@@ -1685,15 +1754,15 @@
         <v>420</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" s="9" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A8" s="16">
-        <v>50</v>
+      <c r="A8" s="16" t="s">
+        <v>7</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" s="16">
         <v>50</v>
@@ -1708,15 +1777,15 @@
         <v>440</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" s="10" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A9" s="18">
-        <v>55</v>
+      <c r="A9" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C9" s="18">
         <v>55</v>
@@ -1731,15 +1800,15 @@
         <v>330</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" s="10" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A10" s="18">
-        <v>55</v>
+      <c r="A10" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10" s="18">
         <v>55</v>
@@ -1754,15 +1823,15 @@
         <v>350</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" s="10" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A11" s="18">
-        <v>55</v>
+      <c r="A11" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C11" s="18">
         <v>55</v>
@@ -1777,15 +1846,15 @@
         <v>370</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" s="10" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A12" s="18">
-        <v>55</v>
+      <c r="A12" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C12" s="18">
         <v>55</v>
@@ -1800,15 +1869,15 @@
         <v>390</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" s="10" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A13" s="18">
-        <v>55</v>
+      <c r="A13" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C13" s="18">
         <v>55</v>
@@ -1823,15 +1892,15 @@
         <v>410</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" s="10" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A14" s="18">
-        <v>55</v>
+      <c r="A14" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C14" s="18">
         <v>55</v>
@@ -1846,15 +1915,15 @@
         <v>430</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" s="10" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A15" s="18">
-        <v>55</v>
+      <c r="A15" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C15" s="18">
         <v>55</v>
@@ -1869,15 +1938,15 @@
         <v>450</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" s="11" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A16" s="19">
-        <v>60</v>
+      <c r="A16" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C16" s="19">
         <v>60</v>
@@ -1892,15 +1961,15 @@
         <v>350</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" s="11" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A17" s="19">
-        <v>60</v>
+      <c r="A17" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C17" s="19">
         <v>60</v>
@@ -1915,15 +1984,15 @@
         <v>370</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" s="11" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A18" s="19">
-        <v>60</v>
+      <c r="A18" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C18" s="19">
         <v>60</v>
@@ -1938,15 +2007,15 @@
         <v>390</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" s="11" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A19" s="19">
-        <v>60</v>
+      <c r="A19" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C19" s="19">
         <v>60</v>
@@ -1961,15 +2030,15 @@
         <v>410</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" s="11" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A20" s="19">
-        <v>60</v>
+      <c r="A20" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C20" s="19">
         <v>60</v>
@@ -1984,15 +2053,15 @@
         <v>430</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" s="11" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A21" s="19">
-        <v>60</v>
+      <c r="A21" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C21" s="19">
         <v>60</v>
@@ -2007,15 +2076,15 @@
         <v>450</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" s="11" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A22" s="19">
-        <v>60</v>
+      <c r="A22" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C22" s="19">
         <v>60</v>
@@ -2030,15 +2099,15 @@
         <v>470</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" s="12" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A23" s="20">
-        <v>65</v>
+      <c r="A23" s="20" t="s">
+        <v>37</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C23" s="20">
         <v>65</v>
@@ -2053,15 +2122,15 @@
         <v>360</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" s="12" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A24" s="20">
-        <v>65</v>
+      <c r="A24" s="20" t="s">
+        <v>37</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C24" s="20">
         <v>65</v>
@@ -2076,15 +2145,15 @@
         <v>380</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" s="12" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A25" s="20">
-        <v>65</v>
+      <c r="A25" s="20" t="s">
+        <v>37</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C25" s="20">
         <v>65</v>
@@ -2099,15 +2168,15 @@
         <v>400</v>
       </c>
       <c r="G25" s="17" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" s="12" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A26" s="20">
-        <v>65</v>
+      <c r="A26" s="20" t="s">
+        <v>37</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C26" s="20">
         <v>65</v>
@@ -2122,15 +2191,15 @@
         <v>420</v>
       </c>
       <c r="G26" s="17" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" s="12" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A27" s="20">
-        <v>65</v>
+      <c r="A27" s="20" t="s">
+        <v>37</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C27" s="20">
         <v>65</v>
@@ -2145,15 +2214,15 @@
         <v>440</v>
       </c>
       <c r="G27" s="17" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" s="12" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A28" s="20">
-        <v>65</v>
+      <c r="A28" s="20" t="s">
+        <v>37</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C28" s="20">
         <v>65</v>
@@ -2168,15 +2237,15 @@
         <v>460</v>
       </c>
       <c r="G28" s="17" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" s="12" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A29" s="20">
-        <v>65</v>
+      <c r="A29" s="20" t="s">
+        <v>37</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C29" s="20">
         <v>65</v>
@@ -2191,15 +2260,15 @@
         <v>480</v>
       </c>
       <c r="G29" s="17" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="30" s="13" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A30" s="21">
-        <v>70</v>
+      <c r="A30" s="21" t="s">
+        <v>39</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C30" s="21">
         <v>70</v>
@@ -2214,15 +2283,15 @@
         <v>380</v>
       </c>
       <c r="G30" s="17" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" s="13" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A31" s="21">
-        <v>70</v>
+      <c r="A31" s="21" t="s">
+        <v>39</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C31" s="21">
         <v>70</v>
@@ -2237,15 +2306,15 @@
         <v>400</v>
       </c>
       <c r="G31" s="17" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32" s="13" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A32" s="21">
-        <v>70</v>
+      <c r="A32" s="21" t="s">
+        <v>39</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C32" s="21">
         <v>70</v>
@@ -2260,15 +2329,15 @@
         <v>420</v>
       </c>
       <c r="G32" s="17" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" s="13" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A33" s="21">
-        <v>70</v>
+      <c r="A33" s="21" t="s">
+        <v>39</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C33" s="21">
         <v>70</v>
@@ -2283,15 +2352,15 @@
         <v>440</v>
       </c>
       <c r="G33" s="17" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" s="13" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A34" s="21">
-        <v>70</v>
+      <c r="A34" s="21" t="s">
+        <v>39</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C34" s="21">
         <v>70</v>
@@ -2306,15 +2375,15 @@
         <v>460</v>
       </c>
       <c r="G34" s="17" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35" s="13" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A35" s="21">
-        <v>70</v>
+      <c r="A35" s="21" t="s">
+        <v>39</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C35" s="21">
         <v>70</v>
@@ -2329,15 +2398,15 @@
         <v>480</v>
       </c>
       <c r="G35" s="17" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
     </row>
     <row r="36" s="13" customFormat="1" ht="18.75" spans="1:7">
-      <c r="A36" s="22">
-        <v>70</v>
+      <c r="A36" s="21" t="s">
+        <v>39</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C36" s="22">
         <v>70</v>
@@ -2352,7 +2421,7 @@
         <v>500</v>
       </c>
       <c r="G36" s="17" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2377,33 +2446,33 @@
   <sheetData>
     <row r="1" ht="35" customHeight="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7">
       <c r="A2" s="6" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="C2" s="6">
         <v>1.1</v>
@@ -2423,10 +2492,10 @@
     </row>
     <row r="3" customFormat="1" ht="30" customHeight="1" spans="1:7">
       <c r="A3" s="6" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="C3" s="6">
         <v>2.1</v>
@@ -2446,10 +2515,10 @@
     </row>
     <row r="4" customFormat="1" ht="30" customHeight="1" spans="1:7">
       <c r="A4" s="6" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="C4" s="6">
         <v>1.1</v>
@@ -2469,10 +2538,10 @@
     </row>
     <row r="5" customFormat="1" ht="30" customHeight="1" spans="1:7">
       <c r="A5" s="6" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="C5" s="6">
         <v>1.1</v>
@@ -2513,359 +2582,359 @@
   <sheetData>
     <row r="1" ht="15" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>42</v>
+        <v>65</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>